<commit_message>
Add 2025 ICS data, Erik's edits on Lake Mead Conservation program
</commit_message>
<xml_diff>
--- a/AutoReadUSBRData/IntentionallyCreatedSurplus-Summary.xlsx
+++ b/AutoReadUSBRData/IntentionallyCreatedSurplus-Summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rosenberg\Work\USU\Research\ColoradoRiver\RCode\ColoradoRiverCollaborate\LakeMeadWaterConservationProgramAnalysis\ICS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rosenberg\Work\USU\Research\ColoradoRiver\RCode\ColoradoRiverCollaborate\AutoReadUSBRData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31B08831-F21F-417B-B2A4-DC06FFD9E18D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{127F87AD-C3C6-4125-A520-BD70BB88D020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="6" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="80">
   <si>
     <t>Data Sources:</t>
   </si>
@@ -301,6 +301,9 @@
   </si>
   <si>
     <t>Balance - Dec 2024 (AF)</t>
+  </si>
+  <si>
+    <t>Balance - Dec 2025 (AF)</t>
   </si>
 </sst>
 </file>
@@ -448,13 +451,13 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -827,7 +830,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30.7265625" customWidth="1"/>
@@ -911,7 +914,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="2">
-        <f t="shared" ref="F3:F18" si="1">SUM(B3:D3)</f>
+        <f t="shared" ref="F3:F20" si="1">SUM(B3:D3)</f>
         <v>593573</v>
       </c>
       <c r="G3" s="10">
@@ -1251,9 +1254,7 @@
         <f>SUMIFS('By User'!$D$2:$D$43,'By User'!$A$2:$A$43,Balances!$G14,'By User'!$C$2:$C$43,Balances!D$1)</f>
         <v>785913</v>
       </c>
-      <c r="E14" s="2">
-        <v>132975</v>
-      </c>
+      <c r="E14" s="2"/>
       <c r="F14" s="2">
         <f t="shared" si="1"/>
         <v>2312627</v>
@@ -1263,7 +1264,7 @@
       </c>
       <c r="H14" s="11">
         <f>SUM(E14:F14)</f>
-        <v>2445602</v>
+        <v>2312627</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
@@ -1280,19 +1281,18 @@
         <v>865741</v>
       </c>
       <c r="E15" s="16">
-        <f>E14+41000</f>
-        <v>173975</v>
+        <v>159903</v>
       </c>
       <c r="F15" s="2">
-        <f t="shared" si="1"/>
-        <v>2840354</v>
+        <f>SUM(B15:E15)</f>
+        <v>3000257</v>
       </c>
       <c r="G15" s="17">
         <v>2020</v>
       </c>
       <c r="H15" s="11">
         <f>SUM(E15:F15)</f>
-        <v>3014329</v>
+        <v>3160160</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
@@ -1309,22 +1309,21 @@
         <v>949658</v>
       </c>
       <c r="E16" s="16">
-        <f>E15+41000</f>
-        <v>214975</v>
+        <v>163842</v>
       </c>
       <c r="F16" s="2">
-        <f t="shared" si="1"/>
-        <v>2990944</v>
+        <f>SUM(B16:E16)</f>
+        <v>3154786</v>
       </c>
       <c r="G16" s="17">
         <v>2021</v>
       </c>
       <c r="H16" s="11">
         <f>SUM(E16:F16)</f>
-        <v>3205919</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+        <v>3318628</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>58</v>
       </c>
@@ -1338,22 +1337,21 @@
         <v>1038765</v>
       </c>
       <c r="E17" s="16">
-        <f>30000+E16</f>
-        <v>244975</v>
+        <v>134023</v>
       </c>
       <c r="F17" s="2">
-        <f t="shared" si="1"/>
-        <v>3037881</v>
+        <f>SUM(B17:E17)</f>
+        <v>3171904</v>
       </c>
       <c r="G17" s="17">
         <v>2022</v>
       </c>
       <c r="H17" s="11">
         <f>SUM(E17:F17)</f>
-        <v>3282856</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+        <v>3305927</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>59</v>
       </c>
@@ -1364,47 +1362,75 @@
         <v>1661832</v>
       </c>
       <c r="D18" s="21">
-        <v>955543</v>
+        <v>955661</v>
       </c>
       <c r="E18" s="18">
-        <f>E17-34000</f>
-        <v>210975</v>
+        <v>114958</v>
       </c>
       <c r="F18" s="2">
         <f t="shared" si="1"/>
-        <v>3327964</v>
+        <v>3328082</v>
       </c>
       <c r="G18" s="12">
         <v>2023</v>
       </c>
       <c r="H18" s="11">
         <f>SUM(E18:F18)</f>
-        <v>3538939</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+        <v>3443040</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>78</v>
       </c>
-      <c r="B19" s="24">
+      <c r="B19" s="22">
         <v>710589</v>
       </c>
-      <c r="C19" s="24">
+      <c r="C19" s="22">
         <v>1661832</v>
       </c>
-      <c r="D19" s="24">
+      <c r="D19" s="22">
         <v>954013</v>
       </c>
-      <c r="E19" s="24">
-        <v>240975</v>
-      </c>
-      <c r="F19" s="24">
+      <c r="E19" s="22">
+        <v>73529</v>
+      </c>
+      <c r="F19" s="2">
+        <f t="shared" si="1"/>
         <v>3326434</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="12">
         <v>2024</v>
       </c>
-      <c r="H19" s="24">
+      <c r="H19" s="22">
+        <v>3567409</v>
+      </c>
+      <c r="J19" s="22"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" s="16">
+        <v>703050</v>
+      </c>
+      <c r="C20" s="16">
+        <v>1731217</v>
+      </c>
+      <c r="D20" s="16">
+        <v>892864</v>
+      </c>
+      <c r="E20" s="16">
+        <v>132457</v>
+      </c>
+      <c r="F20" s="2">
+        <f>SUM(B20:E20)</f>
+        <v>3459588</v>
+      </c>
+      <c r="G20" s="12">
+        <v>2025</v>
+      </c>
+      <c r="H20" s="22">
         <v>3567409</v>
       </c>
     </row>
@@ -1768,7 +1794,7 @@
       </c>
       <c r="B14" s="16">
         <f t="shared" si="0"/>
-        <v>703670</v>
+        <v>570695</v>
       </c>
       <c r="C14" s="16">
         <f>Balances!B14-Balances!B13</f>
@@ -1784,7 +1810,7 @@
       </c>
       <c r="F14" s="16">
         <f>Balances!E14-Balances!E13</f>
-        <v>132975</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
@@ -1794,7 +1820,7 @@
       </c>
       <c r="B15" s="16">
         <f t="shared" si="0"/>
-        <v>568727</v>
+        <v>687630</v>
       </c>
       <c r="C15" s="16">
         <f>Balances!B15-Balances!B14</f>
@@ -1810,7 +1836,7 @@
       </c>
       <c r="F15" s="16">
         <f>Balances!E15-Balances!E14</f>
-        <v>41000</v>
+        <v>159903</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
@@ -1820,7 +1846,7 @@
       </c>
       <c r="B16" s="16">
         <f t="shared" si="0"/>
-        <v>191590</v>
+        <v>154529</v>
       </c>
       <c r="C16" s="16">
         <f>Balances!B16-Balances!B15</f>
@@ -1836,7 +1862,7 @@
       </c>
       <c r="F16" s="16">
         <f>Balances!E16-Balances!E15</f>
-        <v>41000</v>
+        <v>3939</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
@@ -1846,7 +1872,7 @@
       </c>
       <c r="B17" s="16">
         <f t="shared" si="0"/>
-        <v>76937</v>
+        <v>17118</v>
       </c>
       <c r="C17" s="16">
         <f>Balances!B17-Balances!B16</f>
@@ -1862,7 +1888,7 @@
       </c>
       <c r="F17" s="16">
         <f>Balances!E17-Balances!E16</f>
-        <v>30000</v>
+        <v>-29819</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
@@ -1872,7 +1898,7 @@
       </c>
       <c r="B18" s="16">
         <f t="shared" si="0"/>
-        <v>256083</v>
+        <v>271136</v>
       </c>
       <c r="C18" s="16">
         <f>Balances!B18-Balances!B17</f>
@@ -1884,11 +1910,11 @@
       </c>
       <c r="E18" s="16">
         <f>Balances!D18-Balances!D17</f>
-        <v>-83222</v>
+        <v>-83104</v>
       </c>
       <c r="F18" s="16">
         <f>Balances!E18-Balances!E17</f>
-        <v>-34000</v>
+        <v>-19065</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
@@ -1898,7 +1924,7 @@
       </c>
       <c r="B19" s="16">
         <f t="shared" ref="B19" si="1">SUM(C19:F19)</f>
-        <v>28470</v>
+        <v>-43077</v>
       </c>
       <c r="C19" s="16">
         <f>Balances!B19-Balances!B18</f>
@@ -1910,11 +1936,11 @@
       </c>
       <c r="E19" s="16">
         <f>Balances!D19-Balances!D18</f>
-        <v>-1530</v>
+        <v>-1648</v>
       </c>
       <c r="F19" s="16">
         <f>Balances!E19-Balances!E18</f>
-        <v>30000</v>
+        <v>-41429</v>
       </c>
     </row>
   </sheetData>
@@ -2112,14 +2138,14 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="22"/>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
@@ -2192,11 +2218,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="E1" s="23" t="s">
+      <c r="E1" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
     </row>
     <row r="2" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">

</xml_diff>

<commit_message>
Fix formula error for Mexico in Lake Mead Water Conservation account excel file
</commit_message>
<xml_diff>
--- a/AutoReadUSBRData/IntentionallyCreatedSurplus-Summary.xlsx
+++ b/AutoReadUSBRData/IntentionallyCreatedSurplus-Summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rosenberg\Work\USU\Research\ColoradoRiver\RCode\ColoradoRiverCollaborate\AutoReadUSBRData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{127F87AD-C3C6-4125-A520-BD70BB88D020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F7B8DD1-E311-44DB-A03B-856E7EF848DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="6" r:id="rId1"/>
@@ -914,7 +914,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="2">
-        <f t="shared" ref="F3:F20" si="1">SUM(B3:D3)</f>
+        <f t="shared" ref="F3:F19" si="1">SUM(B3:D3)</f>
         <v>593573</v>
       </c>
       <c r="G3" s="10">
@@ -999,7 +999,6 @@
         <v>482672</v>
       </c>
       <c r="E6" s="2">
-        <f>SUMIFS('By User'!$D$2:$D$43,'By User'!$A$2:$A$43,Balances!$G6,'By User'!$C$2:$C$43,Balances!E$1)</f>
         <v>0</v>
       </c>
       <c r="F6" s="2">
@@ -1031,7 +1030,6 @@
         <v>512804</v>
       </c>
       <c r="E7" s="2">
-        <f>SUMIFS('By User'!$D$2:$D$43,'By User'!$A$2:$A$43,Balances!$G7,'By User'!$C$2:$C$43,Balances!E$1)</f>
         <v>0</v>
       </c>
       <c r="F7" s="2">
@@ -1063,7 +1061,6 @@
         <v>541051</v>
       </c>
       <c r="E8" s="2">
-        <f>SUMIFS('By User'!$D$2:$D$43,'By User'!$A$2:$A$43,Balances!$G8,'By User'!$C$2:$C$43,Balances!E$1)</f>
         <v>0</v>
       </c>
       <c r="F8" s="2">
@@ -1095,7 +1092,6 @@
         <v>564765</v>
       </c>
       <c r="E9" s="2">
-        <f>SUMIFS('By User'!$D$2:$D$43,'By User'!$A$2:$A$43,Balances!$G9,'By User'!$C$2:$C$43,Balances!E$1)</f>
         <v>0</v>
       </c>
       <c r="F9" s="2">
@@ -1127,7 +1123,6 @@
         <v>511023</v>
       </c>
       <c r="E10" s="2">
-        <f>SUMIFS('By User'!$D$2:$D$43,'By User'!$A$2:$A$43,Balances!$G10,'By User'!$C$2:$C$43,Balances!E$1)</f>
         <v>0</v>
       </c>
       <c r="F10" s="2">
@@ -1159,7 +1154,6 @@
         <v>531562</v>
       </c>
       <c r="E11" s="2">
-        <f>SUMIFS('By User'!$D$2:$D$43,'By User'!$A$2:$A$43,Balances!$G11,'By User'!$C$2:$C$43,Balances!E$1)</f>
         <v>0</v>
       </c>
       <c r="F11" s="2">
@@ -1191,7 +1185,6 @@
         <v>582313</v>
       </c>
       <c r="E12" s="2">
-        <f>SUMIFS('By User'!$D$2:$D$43,'By User'!$A$2:$A$43,Balances!$G12,'By User'!$C$2:$C$43,Balances!E$1)</f>
         <v>0</v>
       </c>
       <c r="F12" s="2">
@@ -1223,7 +1216,6 @@
         <v>700448</v>
       </c>
       <c r="E13" s="2">
-        <f>SUMIFS('By User'!$D$2:$D$43,'By User'!$A$2:$A$43,Balances!$G13,'By User'!$C$2:$C$43,Balances!E$1)</f>
         <v>0</v>
       </c>
       <c r="F13" s="2">
@@ -1254,7 +1246,9 @@
         <f>SUMIFS('By User'!$D$2:$D$43,'By User'!$A$2:$A$43,Balances!$G14,'By User'!$C$2:$C$43,Balances!D$1)</f>
         <v>785913</v>
       </c>
-      <c r="E14" s="2"/>
+      <c r="E14" s="2">
+        <v>0</v>
+      </c>
       <c r="F14" s="2">
         <f t="shared" si="1"/>
         <v>2312627</v>

</xml_diff>